<commit_message>
Update keyword data; re-apply billing-period fix
Refresh rileo_data_enrichment.xlsx from the team's export (ruut->rileo
cancel keywords, added reimburst and Spanish patterns, dropped stray
/cancel my account/ from Tech Issue) and re-apply the 'billing period'
negative-lookahead fix that the export had reverted.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rileo_data_enrichment.xlsx
+++ b/rileo_data_enrichment.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D147"/>
+  <dimension ref="A1:D149"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="54.63" customWidth="1" style="15" min="1" max="1"/>
@@ -1259,7 +1259,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>/cancel my subscription to ruut/i,</t>
+          <t>/cancel my subscription to rileo/i,</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>/cancel my account/i,</t>
+          <t>/mobility program add-on/i,</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>/cancel my ruut subscription/i,</t>
+          <t>/cancel my rileo subscription/i,</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -1463,10 +1463,14 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>/cancel all subscriptions to ruut/i,</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="n"/>
+          <t>/cancel all subscriptions to rileo/i,</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>/reimburst/i,</t>
+        </is>
+      </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
           <t>/Mobility Program/i,</t>
@@ -1491,11 +1495,6 @@
           <t>/end my subscription/i,</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>/mobility program add-on/i,</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -1633,7 +1632,7 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>/cancel my subscription for ruut/i,</t>
+          <t>/cancel my subscription for rileo/i,</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1646,7 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>/cancel my ruut subscription/i,</t>
+          <t>/cancel my rileo subscription/i,</t>
         </is>
       </c>
     </row>
@@ -1703,7 +1702,7 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>/ruut account has been canceled/i,</t>
+          <t>/rileo account has been canceled/i,</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1800,7 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>/cancel my subscription with ruut/i,</t>
+          <t>/cancel my subscription with rileo/i,</t>
         </is>
       </c>
     </row>
@@ -1836,7 +1835,7 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>/cancel ruut/i,</t>
+          <t>/cancel rileo/i,</t>
         </is>
       </c>
     </row>
@@ -1885,14 +1884,14 @@
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>/cancel ruut subscription/i,</t>
+          <t>/cancel rileo subscription/i,</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>/cancel my subscription with ruut/i,</t>
+          <t>/cancel my subscription with rileo/i,</t>
         </is>
       </c>
     </row>
@@ -2110,6 +2109,20 @@
       <c r="A147" s="3" t="inlineStr">
         <is>
           <t>/stop my payments/i,</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>/dar de baja (a la )?aplicación/i,</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="4" t="inlineStr">
+        <is>
+          <t>/cancel my account/i,</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update keywords from team (FR/ES cancel, deletion) + reapply billing-period fix
Pulled team's latest data file (+2 cancel patterns for French / Spanish,
+1 Tech Issue pattern 'deletion') and re-applied our local exclusion of
'billing period' from the bill/billing blacklist (negative lookahead),
which the team's export overwrote.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rileo_data_enrichment.xlsx
+++ b/rileo_data_enrichment.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D149"/>
+  <dimension ref="A1:D151"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="54.63" customWidth="1" style="15" min="1" max="1"/>
@@ -1495,6 +1495,11 @@
           <t>/end my subscription/i,</t>
         </is>
       </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>/deletion/i,</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -2123,6 +2128,20 @@
       <c r="A149" s="4" t="inlineStr">
         <is>
           <t>/cancel my account/i,</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="4" t="inlineStr">
+        <is>
+          <t>/annulé mon abonnement/,i</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="4" t="inlineStr">
+        <is>
+          <t>/quiero darme de baja/,i</t>
         </is>
       </c>
     </row>

</xml_diff>